<commit_message>
Added Functionality Testing for E-Commerce
</commit_message>
<xml_diff>
--- a/Assesment_ECommerece_Funcationality Testing.xlsx
+++ b/Assesment_ECommerece_Funcationality Testing.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saurabh Mishra\Downloads\Manual Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46BE929-C90E-4109-889F-F305E4196C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA47ADE-E071-453E-8511-3873A02F3F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D95856B3-4332-434B-9106-A35335285F4A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D95856B3-4332-434B-9106-A35335285F4A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="2" r:id="rId1"/>
-    <sheet name="Product" sheetId="3" r:id="rId2"/>
-    <sheet name="Register" sheetId="1" r:id="rId3"/>
+    <sheet name="Register" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="2" r:id="rId2"/>
+    <sheet name="Product" sheetId="3" r:id="rId3"/>
     <sheet name="Product_Description" sheetId="4" r:id="rId4"/>
     <sheet name="Cart" sheetId="5" r:id="rId5"/>
     <sheet name="Shipping Address" sheetId="6" r:id="rId6"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="235">
   <si>
     <t>SCENARIO_ID</t>
   </si>
@@ -967,7 +967,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1000,18 +1000,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1020,6 +1008,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -1035,7 +1029,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1061,13 +1055,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1381,6 +1371,1010 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFF0423-DAFA-4951-949A-487BA80FCD31}">
+  <dimension ref="A1:D108"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" customWidth="1"/>
+    <col min="3" max="3" width="54.109375" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="14"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="14"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+    </row>
+    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="8"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="8"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="15"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" s="9"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" s="9"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="9"/>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="9"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="9"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="9"/>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="9"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="9"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" s="9"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="9"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" s="9"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="9"/>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" s="9"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="9"/>
+      <c r="D74" s="9"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" s="9"/>
+      <c r="B75" s="9"/>
+      <c r="C75" s="9"/>
+      <c r="D75" s="9"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="9"/>
+      <c r="B76" s="9"/>
+      <c r="C76" s="9"/>
+      <c r="D76" s="9"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="9"/>
+      <c r="B77" s="9"/>
+      <c r="C77" s="9"/>
+      <c r="D77" s="9"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="9"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="9"/>
+      <c r="D78" s="9"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="9"/>
+      <c r="B79" s="9"/>
+      <c r="C79" s="9"/>
+      <c r="D79" s="9"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="9"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
+      <c r="D80" s="9"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="9"/>
+      <c r="B81" s="9"/>
+      <c r="C81" s="9"/>
+      <c r="D81" s="9"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="9"/>
+      <c r="B82" s="9"/>
+      <c r="C82" s="9"/>
+      <c r="D82" s="9"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="9"/>
+      <c r="B83" s="9"/>
+      <c r="C83" s="9"/>
+      <c r="D83" s="9"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="9"/>
+      <c r="B84" s="9"/>
+      <c r="C84" s="9"/>
+      <c r="D84" s="9"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="9"/>
+      <c r="B85" s="9"/>
+      <c r="C85" s="9"/>
+      <c r="D85" s="9"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="9"/>
+      <c r="B86" s="9"/>
+      <c r="C86" s="9"/>
+      <c r="D86" s="9"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="9"/>
+      <c r="B87" s="9"/>
+      <c r="C87" s="9"/>
+      <c r="D87" s="9"/>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="9"/>
+      <c r="B88" s="9"/>
+      <c r="C88" s="9"/>
+      <c r="D88" s="9"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="9"/>
+      <c r="B89" s="9"/>
+      <c r="C89" s="9"/>
+      <c r="D89" s="9"/>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="9"/>
+      <c r="B90" s="9"/>
+      <c r="C90" s="9"/>
+      <c r="D90" s="9"/>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="9"/>
+      <c r="B91" s="9"/>
+      <c r="C91" s="9"/>
+      <c r="D91" s="9"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="9"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="9"/>
+      <c r="D92" s="9"/>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="9"/>
+      <c r="B93" s="9"/>
+      <c r="C93" s="9"/>
+      <c r="D93" s="9"/>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A94" s="9"/>
+      <c r="B94" s="9"/>
+      <c r="C94" s="9"/>
+      <c r="D94" s="9"/>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="9"/>
+      <c r="B95" s="9"/>
+      <c r="C95" s="9"/>
+      <c r="D95" s="9"/>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="9"/>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="9"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" s="9"/>
+      <c r="B97" s="9"/>
+      <c r="C97" s="9"/>
+      <c r="D97" s="9"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" s="9"/>
+      <c r="B98" s="9"/>
+      <c r="C98" s="9"/>
+      <c r="D98" s="9"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A99" s="9"/>
+      <c r="B99" s="9"/>
+      <c r="C99" s="9"/>
+      <c r="D99" s="9"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A100" s="9"/>
+      <c r="B100" s="9"/>
+      <c r="C100" s="9"/>
+      <c r="D100" s="9"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A101" s="9"/>
+      <c r="B101" s="9"/>
+      <c r="C101" s="9"/>
+      <c r="D101" s="9"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A102" s="9"/>
+      <c r="B102" s="9"/>
+      <c r="C102" s="9"/>
+      <c r="D102" s="9"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" s="9"/>
+      <c r="B103" s="9"/>
+      <c r="C103" s="9"/>
+      <c r="D103" s="9"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" s="9"/>
+      <c r="B104" s="9"/>
+      <c r="C104" s="9"/>
+      <c r="D104" s="9"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A105" s="9"/>
+      <c r="B105" s="9"/>
+      <c r="C105" s="9"/>
+      <c r="D105" s="9"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A106" s="9"/>
+      <c r="B106" s="9"/>
+      <c r="C106" s="9"/>
+      <c r="D106" s="9"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A107" s="9"/>
+      <c r="B107" s="9"/>
+      <c r="C107" s="9"/>
+      <c r="D107" s="9"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" s="9"/>
+      <c r="B108" s="9"/>
+      <c r="C108" s="9"/>
+      <c r="D108" s="9"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813C6E1F-F8E0-45A9-8C5E-F95369D058CB}">
   <dimension ref="A2:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1608,7 +2602,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AE38A35-60D7-432F-872A-F1169E9D317B}">
   <dimension ref="A2:D32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1725,10 +2719,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1787,10 +2781,10 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
@@ -1877,10 +2871,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -1897,10 +2891,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
@@ -1925,1014 +2919,6 @@
       <c r="A32" s="5" t="s">
         <v>234</v>
       </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFF0423-DAFA-4951-949A-487BA80FCD31}">
-  <dimension ref="A1:D108"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="30.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" customWidth="1"/>
-    <col min="3" max="3" width="54.109375" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B1" s="17"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="17"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-    </row>
-    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B47" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="12"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C53" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D55" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B56" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12"/>
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="9"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B61" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="9"/>
-      <c r="B62" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="9"/>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="9"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="9"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="9"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="9"/>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="9"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="9"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="9"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="9"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="9"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="9"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="9"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="9"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="D75" s="9"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="9"/>
-      <c r="B76" s="9"/>
-      <c r="C76" s="9"/>
-      <c r="D76" s="9"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="9"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="9"/>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
-      <c r="D78" s="9"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="9"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
-      <c r="D79" s="9"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="9"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="9"/>
-      <c r="D80" s="9"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="9"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
-      <c r="D81" s="9"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="9"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
-      <c r="D82" s="9"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="9"/>
-      <c r="B83" s="9"/>
-      <c r="C83" s="9"/>
-      <c r="D83" s="9"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="9"/>
-      <c r="B84" s="9"/>
-      <c r="C84" s="9"/>
-      <c r="D84" s="9"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="9"/>
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-      <c r="D85" s="9"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="9"/>
-      <c r="B86" s="9"/>
-      <c r="C86" s="9"/>
-      <c r="D86" s="9"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="9"/>
-      <c r="B87" s="9"/>
-      <c r="C87" s="9"/>
-      <c r="D87" s="9"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="9"/>
-      <c r="B88" s="9"/>
-      <c r="C88" s="9"/>
-      <c r="D88" s="9"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="9"/>
-      <c r="B89" s="9"/>
-      <c r="C89" s="9"/>
-      <c r="D89" s="9"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="9"/>
-      <c r="B90" s="9"/>
-      <c r="C90" s="9"/>
-      <c r="D90" s="9"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="9"/>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9"/>
-      <c r="D91" s="9"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="9"/>
-      <c r="B92" s="9"/>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="9"/>
-      <c r="B93" s="9"/>
-      <c r="C93" s="9"/>
-      <c r="D93" s="9"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="9"/>
-      <c r="B94" s="9"/>
-      <c r="C94" s="9"/>
-      <c r="D94" s="9"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="9"/>
-      <c r="B95" s="9"/>
-      <c r="C95" s="9"/>
-      <c r="D95" s="9"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="9"/>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9"/>
-      <c r="D96" s="9"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" s="9"/>
-      <c r="B97" s="9"/>
-      <c r="C97" s="9"/>
-      <c r="D97" s="9"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" s="9"/>
-      <c r="B98" s="9"/>
-      <c r="C98" s="9"/>
-      <c r="D98" s="9"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="9"/>
-      <c r="B99" s="9"/>
-      <c r="C99" s="9"/>
-      <c r="D99" s="9"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="9"/>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9"/>
-      <c r="D100" s="9"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="9"/>
-      <c r="B101" s="9"/>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="9"/>
-      <c r="B102" s="9"/>
-      <c r="C102" s="9"/>
-      <c r="D102" s="9"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="9"/>
-      <c r="B103" s="9"/>
-      <c r="C103" s="9"/>
-      <c r="D103" s="9"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="9"/>
-      <c r="B104" s="9"/>
-      <c r="C104" s="9"/>
-      <c r="D104" s="9"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A105" s="9"/>
-      <c r="B105" s="9"/>
-      <c r="C105" s="9"/>
-      <c r="D105" s="9"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106" s="9"/>
-      <c r="B106" s="9"/>
-      <c r="C106" s="9"/>
-      <c r="D106" s="9"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="9"/>
-      <c r="B107" s="9"/>
-      <c r="C107" s="9"/>
-      <c r="D107" s="9"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="9"/>
-      <c r="B108" s="9"/>
-      <c r="C108" s="9"/>
-      <c r="D108" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -3030,10 +3016,10 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3126,16 +3112,16 @@
       <c r="D18" s="3"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3622,16 +3608,16 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="14" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>